<commit_message>
Updating the coordinates for the sites
</commit_message>
<xml_diff>
--- a/Jones_honours/01_raw_data/RLS_CANADA_Bamfield_2021.xlsx
+++ b/Jones_honours/01_raw_data/RLS_CANADA_Bamfield_2021.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alecjones/Documents/GitHub/Alec_Jones_Honours/Jones_honours/01_raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D49540-2723-C24B-B5AE-FFEDC7B09620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C279271B-B442-2446-BABB-176737D5FB47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5560" yWindow="22500" windowWidth="27380" windowHeight="14240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28080" yWindow="4440" windowWidth="27380" windowHeight="14240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SUMMARY" sheetId="13" state="hidden" r:id="rId1"/>

</xml_diff>

<commit_message>
Showing plots in meeting
</commit_message>
<xml_diff>
--- a/Jones_honours/01_raw_data/RLS_CANADA_Bamfield_2021.xlsx
+++ b/Jones_honours/01_raw_data/RLS_CANADA_Bamfield_2021.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alecjones/Documents/GitHub/Alec_Jones_Honours/Jones_honours/01_raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C279271B-B442-2446-BABB-176737D5FB47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AF67E4A-40C1-554A-BC8A-4499D7CACF93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28080" yWindow="4440" windowWidth="27380" windowHeight="14240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4960" yWindow="1340" windowWidth="27380" windowHeight="14240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SUMMARY" sheetId="13" state="hidden" r:id="rId1"/>

</xml_diff>

<commit_message>
Working on getting all years data
</commit_message>
<xml_diff>
--- a/Jones_honours/01_raw_data/RLS_CANADA_Bamfield_2021.xlsx
+++ b/Jones_honours/01_raw_data/RLS_CANADA_Bamfield_2021.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alecjones/Documents/GitHub/Alec_Jones_Honours/Jones_honours/01_raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AF67E4A-40C1-554A-BC8A-4499D7CACF93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE5594CA-E60D-4E45-810C-0A9030419350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4960" yWindow="1340" windowWidth="27380" windowHeight="14240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1080" yWindow="900" windowWidth="27380" windowHeight="14260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SUMMARY" sheetId="13" state="hidden" r:id="rId1"/>
@@ -29,8 +29,8 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="158" r:id="rId9"/>
-    <pivotCache cacheId="159" r:id="rId10"/>
+    <pivotCache cacheId="4" r:id="rId9"/>
+    <pivotCache cacheId="5" r:id="rId10"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -3316,7 +3316,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable1" cacheId="158" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="4" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="1" indent="0" compact="0" compactData="0" gridDropZones="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable1" cacheId="4" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="4" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="1" indent="0" compact="0" compactData="0" gridDropZones="1">
   <location ref="A3:E46" firstHeaderRow="1" firstDataRow="4" firstDataCol="2"/>
   <pivotFields count="18">
     <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>
@@ -3564,7 +3564,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0700-000001000000}" name="PivotTable2" cacheId="159" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="5" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="1" indent="0" compact="0" compactData="0" gridDropZones="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0700-000001000000}" name="PivotTable2" cacheId="5" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="5" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="1" indent="0" compact="0" compactData="0" gridDropZones="1">
   <location ref="A3:I8" firstHeaderRow="1" firstDataRow="2" firstDataCol="6"/>
   <pivotFields count="48">
     <pivotField compact="0" outline="0" subtotalTop="0" showAll="0" includeNewItemsInFilter="1"/>

</xml_diff>